<commit_message>
jalar los asientos al reporte diario
</commit_message>
<xml_diff>
--- a/public/reporte_lcaja.xlsx
+++ b/public/reporte_lcaja.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="46">
   <si>
     <t>SALDO ANT</t>
   </si>
@@ -47,7 +47,7 @@
     <t>CAJA</t>
   </si>
   <si>
-    <t>2025-10-10</t>
+    <t>2025-04-05</t>
   </si>
   <si>
     <t>Ingreso</t>
@@ -56,67 +56,103 @@
     <t>Haber</t>
   </si>
   <si>
-    <t>Facturas, boletas y otros comprobantes por cobrar</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-6, 18838574 DANIEL IZQUIERDO</t>
+    <t>Diezmo actual</t>
+  </si>
+  <si>
+    <t>POR DIEZMO FECHA 05-04-2025</t>
   </si>
   <si>
     <t>Principal</t>
   </si>
   <si>
-    <t>BOLETA EB01-7, 18838574 DANIEL IZQUIERDO DIEZMO Y OFRENDA</t>
-  </si>
-  <si>
-    <t>2025-10-24</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-8, 47329849 KEVIN ENRIQUE LOYOLA MERCADO</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-9, 70652190 JESUS MANUEL GUTIERREZ ARENAS</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-10, 18898317 ALBERTO ELEUTERIO ORTIZ CRUZ</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-11, 18837971 JUANA BERTHA JUAREZ DE LA CRUZ</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-12, 76083131 JONATHAN RUBEN RAMIREZ SANGAY</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-13, 42231190 JULIO RUBEN RAMIREZ PABLO</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-14, 18861304 ALIPIO ANTONIO AVILA VALENCIA</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-15, 18848453 JAIME  LUIS CORCUERA UCEDA</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-16, 99999999 OFRENDAS LIBRES</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-17, 75495571 EVELYN MARGARITA MEZA RUIZ</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-18, 18837961JORGE ALBERTO GARCIA JUAREZ</t>
-  </si>
-  <si>
-    <t>BOLETA EB01-19, 99999999 APORTE LIBRE</t>
-  </si>
-  <si>
     <t>Egreso</t>
   </si>
   <si>
     <t>Debe</t>
   </si>
   <si>
+    <t>Gastos varios</t>
+  </si>
+  <si>
+    <t>OFRENDA MISIONERA</t>
+  </si>
+  <si>
+    <t>2025-04-07</t>
+  </si>
+  <si>
+    <t>POR DIEZMO FECHA 07-04-2025</t>
+  </si>
+  <si>
+    <t>Otras remuneraciones-labores varias</t>
+  </si>
+  <si>
+    <t>OFRENDA DE AMOR A HNO EVER BAZAN</t>
+  </si>
+  <si>
+    <t>OFRENDA DE AMOR A HNO NELSON MUDARRA</t>
+  </si>
+  <si>
+    <t>OFRENDA DE AMOR A HNO SEGUNDO</t>
+  </si>
+  <si>
+    <t>Servicios básicos, agua luz</t>
+  </si>
+  <si>
+    <t>PAGO DE LUZ</t>
+  </si>
+  <si>
+    <t>2025-04-10</t>
+  </si>
+  <si>
+    <t>DIEZMO EVER BAZAN Y FAMILIA</t>
+  </si>
+  <si>
+    <t>2025-04-11</t>
+  </si>
+  <si>
+    <t>DIEZMO NELSON MUDARRA Y FAMILIA</t>
+  </si>
+  <si>
+    <t>Transporte y gastos de viaje</t>
+  </si>
+  <si>
+    <t>POR PASAJE A LIMA A HNO ALBERTO IZQUIERDO</t>
+  </si>
+  <si>
+    <t>POR PASAJE A LIMA A HNO NELSON MUDARRA</t>
+  </si>
+  <si>
+    <t>2025-04-15</t>
+  </si>
+  <si>
+    <t>POR DIEZMO FECHA 15-04-2025</t>
+  </si>
+  <si>
+    <t>2025-04-17</t>
+  </si>
+  <si>
+    <t>OFRENDA DE AMOR A HNO ALBERTO ORTIZ</t>
+  </si>
+  <si>
+    <t>2025-04-23</t>
+  </si>
+  <si>
     <t>Ctas x Pagar-fact. Compras, R/luz</t>
   </si>
   <si>
-    <t>FACTURA F001, 20609912937 COMPRA TECLADO</t>
+    <t>FACTURA F001-1774, 20482360140</t>
+  </si>
+  <si>
+    <t>2025-04-28</t>
+  </si>
+  <si>
+    <t>POR COMBUSTIBLE</t>
+  </si>
+  <si>
+    <t>2025-04-30</t>
+  </si>
+  <si>
+    <t>APOYO A OFRENDA MISIONERA</t>
   </si>
 </sst>
 </file>
@@ -456,17 +492,17 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="4.57" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="22.28" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="9.283" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="6.998" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="4.57" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="58.843" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="68.269" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="42.418" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="49.417" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="11.711" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
@@ -475,7 +511,7 @@
         <v>0</v>
       </c>
       <c r="C1">
-        <v>136.099999999999994</v>
+        <v>694.29999999999995</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -515,7 +551,7 @@
         <v>10</v>
       </c>
       <c r="C4">
-        <v>20.0</v>
+        <v>942.79999999999995</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -524,7 +560,7 @@
         <v>12</v>
       </c>
       <c r="F4">
-        <v>121</v>
+        <v>751</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -544,22 +580,22 @@
         <v>10</v>
       </c>
       <c r="C5">
-        <v>18.0</v>
+        <v>200.0</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F5">
-        <v>121</v>
+        <v>654</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I5" t="s">
         <v>15</v>
@@ -570,10 +606,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C6">
-        <v>500.0</v>
+        <v>17.0</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
@@ -582,13 +618,13 @@
         <v>12</v>
       </c>
       <c r="F6">
-        <v>121</v>
+        <v>751</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
       </c>
       <c r="H6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I6" t="s">
         <v>15</v>
@@ -599,10 +635,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C7">
-        <v>500.0</v>
+        <v>19.0</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -611,13 +647,13 @@
         <v>12</v>
       </c>
       <c r="F7">
-        <v>121</v>
+        <v>751</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
       </c>
       <c r="H7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I7" t="s">
         <v>15</v>
@@ -628,25 +664,25 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>505.0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
         <v>17</v>
       </c>
-      <c r="C8">
-        <v>500.0</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
       <c r="F8">
-        <v>121</v>
+        <v>622</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I8" t="s">
         <v>15</v>
@@ -657,25 +693,25 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9">
+        <v>202.0</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s">
         <v>17</v>
       </c>
-      <c r="C9">
-        <v>500.0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
       <c r="F9">
-        <v>121</v>
+        <v>622</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I9" t="s">
         <v>15</v>
@@ -686,25 +722,25 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10">
+        <v>200.0</v>
+      </c>
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" t="s">
         <v>17</v>
       </c>
-      <c r="C10">
-        <v>500.0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
       <c r="F10">
-        <v>121</v>
+        <v>622</v>
       </c>
       <c r="G10" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I10" t="s">
         <v>15</v>
@@ -715,25 +751,25 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <v>34.4</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
         <v>17</v>
       </c>
-      <c r="C11">
-        <v>500.0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
       <c r="F11">
-        <v>121</v>
+        <v>636</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="H11" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="I11" t="s">
         <v>15</v>
@@ -744,10 +780,10 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C12">
-        <v>250.0</v>
+        <v>300.0</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -756,13 +792,13 @@
         <v>12</v>
       </c>
       <c r="F12">
-        <v>121</v>
+        <v>751</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
       </c>
       <c r="H12" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I12" t="s">
         <v>15</v>
@@ -773,10 +809,10 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C13">
-        <v>250.0</v>
+        <v>50.0</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -785,13 +821,13 @@
         <v>12</v>
       </c>
       <c r="F13">
-        <v>121</v>
+        <v>751</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="I13" t="s">
         <v>15</v>
@@ -802,25 +838,25 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14">
+        <v>200.0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" t="s">
         <v>17</v>
       </c>
-      <c r="C14">
-        <v>500.0</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>12</v>
-      </c>
       <c r="F14">
-        <v>121</v>
+        <v>631</v>
       </c>
       <c r="G14" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="H14" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="I14" t="s">
         <v>15</v>
@@ -831,25 +867,25 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15">
+        <v>200.0</v>
+      </c>
+      <c r="D15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" t="s">
         <v>17</v>
       </c>
-      <c r="C15">
-        <v>500.0</v>
-      </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>12</v>
-      </c>
       <c r="F15">
-        <v>121</v>
+        <v>631</v>
       </c>
       <c r="G15" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="H15" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="I15" t="s">
         <v>15</v>
@@ -860,10 +896,10 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="C16">
-        <v>500.0</v>
+        <v>140.0</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -872,13 +908,13 @@
         <v>12</v>
       </c>
       <c r="F16">
-        <v>121</v>
+        <v>751</v>
       </c>
       <c r="G16" t="s">
         <v>13</v>
       </c>
       <c r="H16" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="I16" t="s">
         <v>15</v>
@@ -889,10 +925,10 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="C17">
-        <v>480.0</v>
+        <v>28.0</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -901,13 +937,13 @@
         <v>12</v>
       </c>
       <c r="F17">
-        <v>121</v>
+        <v>751</v>
       </c>
       <c r="G17" t="s">
         <v>13</v>
       </c>
       <c r="H17" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="I17" t="s">
         <v>15</v>
@@ -918,27 +954,143 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18">
+        <v>28.0</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18">
+        <v>751</v>
+      </c>
+      <c r="G18" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" t="s">
+        <v>36</v>
+      </c>
+      <c r="I18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19">
+        <v>16</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19">
+        <v>30.0</v>
+      </c>
+      <c r="D19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" t="s">
         <v>17</v>
       </c>
-      <c r="C18">
-        <v>5480.0</v>
-      </c>
-      <c r="D18" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18">
+      <c r="F19">
+        <v>654</v>
+      </c>
+      <c r="G19" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19" t="s">
+        <v>38</v>
+      </c>
+      <c r="I19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20">
+        <v>17</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20">
+        <v>102.5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20">
         <v>421</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G20" t="s">
+        <v>40</v>
+      </c>
+      <c r="H20" t="s">
+        <v>41</v>
+      </c>
+      <c r="I20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21">
+        <v>54.0</v>
+      </c>
+      <c r="D21" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21">
+        <v>631</v>
+      </c>
+      <c r="G21" t="s">
         <v>32</v>
       </c>
-      <c r="H18" t="s">
-        <v>33</v>
-      </c>
-      <c r="I18" t="s">
+      <c r="H21" t="s">
+        <v>43</v>
+      </c>
+      <c r="I21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22">
+        <v>19</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22">
+        <v>202.0</v>
+      </c>
+      <c r="D22" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22">
+        <v>654</v>
+      </c>
+      <c r="G22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H22" t="s">
+        <v>45</v>
+      </c>
+      <c r="I22" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>